<commit_message>
feat: implement database configuration management, bulk leave processing, and release automation tools
</commit_message>
<xml_diff>
--- a/templates/Bring_Forward_Template.xlsx
+++ b/templates/Bring_Forward_Template.xlsx
@@ -1,75 +1,83 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
-  <sheets>
-    <sheet state="visible" name="BF" sheetId="1" r:id="rId5"/>
-  </sheets>
-  <definedNames/>
-  <calcPr/>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BF" sheetId="1" r:id="Rec9f383eed10458f"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t xml:space="preserve">Employee Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Employee Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remark</t>
-  </si>
-</sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
-    <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font/>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="lightGray"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border/>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
-  </cellStyles>
-  <dxfs count="0"/>
-</styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:fonts count="3">
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font/>
+    <x:font>
+      <x:b/>
+      <x:color rgb="FFFFFFFF"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="3">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="lightGray"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4D78"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="2">
+    <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C2CC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C2CC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C2CC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C2CC"/>
+      </x:bottom>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="6">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -109,19 +117,19 @@
         <a:srgbClr val="1155CC"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Sheets">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -130,23 +138,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -156,23 +164,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -180,26 +188,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -234,17 +239,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -263,24 +268,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:cols>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Employee Code</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Employee Name</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Bring Forward Days</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Credit Leave Days</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>